<commit_message>
Mise à jour FRLMEnrty 875d09599692a31095fad110c27896c4cb7b25cb
</commit_message>
<xml_diff>
--- a/ML-Entrees/ig/StructureDefinition-fr-lm-allergy-intolerance.xlsx
+++ b/ML-Entrees/ig/StructureDefinition-fr-lm-allergy-intolerance.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="203">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-07T10:50:27+00:00</t>
+    <t>2026-04-07T13:39:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -295,21 +295,48 @@
     <t>fr-lm-allergy-intolerance.header.author[x]</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-personne-structure
-https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-systeme-structure-auteur</t>
-  </si>
-  <si>
-    <t>Auteur(s) responsable(s) : Personne(s) ayant la responsabilité des informations fournies. Le rôle précis de l’auteur responsable dépend du contexte d’usage et du modèle concerné.</t>
+    <t>author[x] peut correspondre soit à un professionnel, soit à une organisation, soit à un système.</t>
   </si>
   <si>
     <t>fr-lm-entry.header.author[x]</t>
   </si>
   <si>
-    <t>fr-lm-allergy-intolerance.header.performer</t>
+    <t>fr-lm-allergy-intolerance.header.author[x].authorProfessional</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-personne-structure
 </t>
+  </si>
+  <si>
+    <t>L'auteur est un professionnel de santé</t>
+  </si>
+  <si>
+    <t>fr-lm-entry.header.author[x].authorProfessional</t>
+  </si>
+  <si>
+    <t>fr-lm-allergy-intolerance.header.author[x].authorOrganisation</t>
+  </si>
+  <si>
+    <t>L'auteur est une organisation</t>
+  </si>
+  <si>
+    <t>fr-lm-entry.header.author[x].authorOrganisation</t>
+  </si>
+  <si>
+    <t>fr-lm-allergy-intolerance.header.author[x].authorDevice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-systeme-structure-auteur
+</t>
+  </si>
+  <si>
+    <t>L'auteur est un système</t>
+  </si>
+  <si>
+    <t>fr-lm-entry.header.author[x].authorDevice</t>
+  </si>
+  <si>
+    <t>fr-lm-allergy-intolerance.header.performer</t>
   </si>
   <si>
     <t>Exécutant (performer)</t>
@@ -924,11 +951,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ37"/>
+  <dimension ref="A1:AJ40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="41.06640625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="41.06640625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="49.61328125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="49.61328125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="10.83984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -1502,13 +1529,13 @@
         <v>73</v>
       </c>
       <c r="K6" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="L6" t="s" s="2">
         <v>92</v>
       </c>
-      <c r="L6" t="s" s="2">
-        <v>93</v>
-      </c>
       <c r="M6" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1559,7 +1586,7 @@
         <v>73</v>
       </c>
       <c r="AF6" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>74</v>
@@ -1576,10 +1603,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1602,13 +1629,13 @@
         <v>73</v>
       </c>
       <c r="K7" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="L7" t="s" s="2">
         <v>96</v>
       </c>
-      <c r="L7" t="s" s="2">
-        <v>97</v>
-      </c>
       <c r="M7" t="s" s="2">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1659,7 +1686,7 @@
         <v>73</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>74</v>
@@ -1676,10 +1703,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1702,13 +1729,13 @@
         <v>73</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1759,7 +1786,7 @@
         <v>73</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>74</v>
@@ -1776,10 +1803,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1802,13 +1829,13 @@
         <v>73</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1859,7 +1886,7 @@
         <v>73</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>74</v>
@@ -1876,10 +1903,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1890,7 +1917,7 @@
         <v>74</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>73</v>
@@ -1902,13 +1929,13 @@
         <v>73</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1959,13 +1986,13 @@
         <v>73</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI10" t="s" s="2">
         <v>73</v>
@@ -1976,10 +2003,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -1990,7 +2017,7 @@
         <v>74</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H11" t="s" s="2">
         <v>73</v>
@@ -2002,13 +2029,13 @@
         <v>73</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2059,13 +2086,13 @@
         <v>73</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH11" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI11" t="s" s="2">
         <v>73</v>
@@ -2076,10 +2103,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2090,7 +2117,7 @@
         <v>74</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>73</v>
@@ -2102,13 +2129,13 @@
         <v>73</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2159,13 +2186,13 @@
         <v>73</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI12" t="s" s="2">
         <v>73</v>
@@ -2176,10 +2203,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2187,7 +2214,7 @@
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s" s="2">
         <v>79</v>
@@ -2202,13 +2229,13 @@
         <v>73</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2238,10 +2265,10 @@
         <v>73</v>
       </c>
       <c r="Y13" t="s" s="2">
-        <v>120</v>
+        <v>73</v>
       </c>
       <c r="Z13" t="s" s="2">
-        <v>121</v>
+        <v>73</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>73</v>
@@ -2259,10 +2286,10 @@
         <v>73</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AG13" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH13" t="s" s="2">
         <v>79</v>
@@ -2276,10 +2303,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2287,7 +2314,7 @@
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G14" t="s" s="2">
         <v>79</v>
@@ -2302,13 +2329,13 @@
         <v>73</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2359,10 +2386,10 @@
         <v>73</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AG14" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH14" t="s" s="2">
         <v>79</v>
@@ -2387,7 +2414,7 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>79</v>
@@ -2402,7 +2429,7 @@
         <v>73</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="L15" t="s" s="2">
         <v>125</v>
@@ -2459,10 +2486,10 @@
         <v>73</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="AG15" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH15" t="s" s="2">
         <v>79</v>
@@ -2476,10 +2503,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2487,7 +2514,7 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G16" t="s" s="2">
         <v>79</v>
@@ -2502,7 +2529,7 @@
         <v>73</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="L16" t="s" s="2">
         <v>128</v>
@@ -2538,10 +2565,10 @@
         <v>73</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>73</v>
@@ -2559,10 +2586,10 @@
         <v>73</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AG16" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH16" t="s" s="2">
         <v>79</v>
@@ -2576,10 +2603,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2587,7 +2614,7 @@
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G17" t="s" s="2">
         <v>79</v>
@@ -2602,13 +2629,13 @@
         <v>73</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2638,31 +2665,31 @@
         <v>73</v>
       </c>
       <c r="Y17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="Z17" t="s" s="2">
-        <v>132</v>
-      </c>
-      <c r="AA17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>129</v>
-      </c>
       <c r="AG17" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH17" t="s" s="2">
         <v>79</v>
@@ -2687,7 +2714,7 @@
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G18" t="s" s="2">
         <v>79</v>
@@ -2702,7 +2729,7 @@
         <v>73</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="L18" t="s" s="2">
         <v>134</v>
@@ -2738,10 +2765,10 @@
         <v>73</v>
       </c>
       <c r="Y18" t="s" s="2">
-        <v>135</v>
+        <v>73</v>
       </c>
       <c r="Z18" t="s" s="2">
-        <v>136</v>
+        <v>73</v>
       </c>
       <c r="AA18" t="s" s="2">
         <v>73</v>
@@ -2762,7 +2789,7 @@
         <v>133</v>
       </c>
       <c r="AG18" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH18" t="s" s="2">
         <v>79</v>
@@ -2776,10 +2803,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2802,13 +2829,13 @@
         <v>73</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2838,10 +2865,10 @@
         <v>73</v>
       </c>
       <c r="Y19" t="s" s="2">
-        <v>139</v>
+        <v>73</v>
       </c>
       <c r="Z19" t="s" s="2">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>73</v>
@@ -2859,7 +2886,7 @@
         <v>73</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>74</v>
@@ -2876,10 +2903,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2887,7 +2914,7 @@
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G20" t="s" s="2">
         <v>79</v>
@@ -2902,13 +2929,13 @@
         <v>73</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2938,10 +2965,10 @@
         <v>73</v>
       </c>
       <c r="Y20" t="s" s="2">
-        <v>73</v>
+        <v>140</v>
       </c>
       <c r="Z20" t="s" s="2">
-        <v>73</v>
+        <v>141</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>73</v>
@@ -2959,10 +2986,10 @@
         <v>73</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="AG20" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH20" t="s" s="2">
         <v>79</v>
@@ -2971,15 +2998,15 @@
         <v>73</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>144</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3002,13 +3029,13 @@
         <v>73</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3038,10 +3065,10 @@
         <v>73</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>73</v>
+        <v>144</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>73</v>
+        <v>145</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>73</v>
@@ -3059,7 +3086,7 @@
         <v>73</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>74</v>
@@ -3076,21 +3103,21 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>150</v>
+        <v>73</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>73</v>
@@ -3102,17 +3129,15 @@
         <v>73</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>154</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>73</v>
@@ -3140,48 +3165,48 @@
         <v>73</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>73</v>
+        <v>148</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>73</v>
+        <v>149</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>155</v>
+        <v>73</v>
       </c>
       <c r="AC22" t="s" s="2">
-        <v>156</v>
+        <v>73</v>
       </c>
       <c r="AD22" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>157</v>
+        <v>73</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>144</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3204,17 +3229,15 @@
         <v>73</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>163</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>73</v>
@@ -3263,7 +3286,7 @@
         <v>73</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>79</v>
@@ -3275,15 +3298,15 @@
         <v>73</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3306,13 +3329,13 @@
         <v>73</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3363,7 +3386,7 @@
         <v>73</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>74</v>
@@ -3375,26 +3398,26 @@
         <v>73</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>170</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>73</v>
@@ -3406,15 +3429,17 @@
         <v>73</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>108</v>
+        <v>160</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>163</v>
+      </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>73</v>
@@ -3451,39 +3476,39 @@
         <v>73</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>73</v>
+        <v>164</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>73</v>
+        <v>166</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3491,7 +3516,7 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
         <v>79</v>
@@ -3506,15 +3531,17 @@
         <v>73</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>108</v>
+        <v>169</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N26" s="2"/>
+        <v>171</v>
+      </c>
+      <c r="N26" t="s" s="2">
+        <v>172</v>
+      </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>73</v>
@@ -3566,7 +3593,7 @@
         <v>173</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH26" t="s" s="2">
         <v>79</v>
@@ -3580,10 +3607,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3594,7 +3621,7 @@
         <v>74</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>73</v>
@@ -3606,13 +3633,13 @@
         <v>73</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="L27" t="s" s="2">
         <v>176</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3663,27 +3690,27 @@
         <v>73</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>73</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3706,13 +3733,13 @@
         <v>73</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3742,7 +3769,7 @@
         <v>73</v>
       </c>
       <c r="Y28" t="s" s="2">
-        <v>179</v>
+        <v>73</v>
       </c>
       <c r="Z28" t="s" s="2">
         <v>73</v>
@@ -3763,7 +3790,7 @@
         <v>73</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>74</v>
@@ -3780,10 +3807,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3791,7 +3818,7 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G29" t="s" s="2">
         <v>79</v>
@@ -3806,13 +3833,13 @@
         <v>73</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -3842,31 +3869,31 @@
         <v>73</v>
       </c>
       <c r="Y29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE29" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF29" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="Z29" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AA29" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB29" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC29" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD29" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE29" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF29" t="s" s="2">
-        <v>180</v>
-      </c>
       <c r="AG29" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH29" t="s" s="2">
         <v>79</v>
@@ -3880,10 +3907,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -3894,7 +3921,7 @@
         <v>74</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>73</v>
@@ -3906,13 +3933,13 @@
         <v>73</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -3942,10 +3969,10 @@
         <v>73</v>
       </c>
       <c r="Y30" t="s" s="2">
-        <v>185</v>
+        <v>73</v>
       </c>
       <c r="Z30" t="s" s="2">
-        <v>186</v>
+        <v>73</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>73</v>
@@ -3963,13 +3990,13 @@
         <v>73</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>73</v>
@@ -3980,10 +4007,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -3991,7 +4018,7 @@
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>79</v>
@@ -4006,13 +4033,13 @@
         <v>73</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>143</v>
+        <v>187</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>143</v>
+        <v>187</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4042,7 +4069,7 @@
         <v>73</v>
       </c>
       <c r="Y31" t="s" s="2">
-        <v>73</v>
+        <v>188</v>
       </c>
       <c r="Z31" t="s" s="2">
         <v>73</v>
@@ -4063,10 +4090,10 @@
         <v>73</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AG31" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH31" t="s" s="2">
         <v>79</v>
@@ -4075,15 +4102,15 @@
         <v>73</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>144</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4091,7 +4118,7 @@
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G32" t="s" s="2">
         <v>79</v>
@@ -4106,13 +4133,13 @@
         <v>73</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>146</v>
+        <v>190</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>147</v>
+        <v>190</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4142,7 +4169,7 @@
         <v>73</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>73</v>
+        <v>191</v>
       </c>
       <c r="Z32" t="s" s="2">
         <v>73</v>
@@ -4163,10 +4190,10 @@
         <v>73</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>148</v>
+        <v>189</v>
       </c>
       <c r="AG32" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH32" t="s" s="2">
         <v>79</v>
@@ -4180,21 +4207,21 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>150</v>
+        <v>73</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>73</v>
@@ -4206,17 +4233,15 @@
         <v>73</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>152</v>
+        <v>193</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>154</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>73</v>
@@ -4244,48 +4269,48 @@
         <v>73</v>
       </c>
       <c r="Y33" t="s" s="2">
-        <v>73</v>
+        <v>194</v>
       </c>
       <c r="Z33" t="s" s="2">
-        <v>73</v>
+        <v>195</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>155</v>
+        <v>73</v>
       </c>
       <c r="AC33" t="s" s="2">
-        <v>156</v>
+        <v>73</v>
       </c>
       <c r="AD33" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>157</v>
+        <v>73</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>144</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4308,17 +4333,15 @@
         <v>73</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>163</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>73</v>
@@ -4367,7 +4390,7 @@
         <v>73</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>164</v>
+        <v>196</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -4379,15 +4402,15 @@
         <v>73</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4410,13 +4433,13 @@
         <v>73</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -4467,7 +4490,7 @@
         <v>73</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>74</v>
@@ -4479,26 +4502,26 @@
         <v>73</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>170</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>73</v>
@@ -4510,15 +4533,17 @@
         <v>73</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>108</v>
+        <v>160</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N36" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="N36" t="s" s="2">
+        <v>163</v>
+      </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>73</v>
@@ -4555,39 +4580,39 @@
         <v>73</v>
       </c>
       <c r="AB36" t="s" s="2">
-        <v>73</v>
+        <v>164</v>
       </c>
       <c r="AC36" t="s" s="2">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="AD36" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE36" t="s" s="2">
-        <v>73</v>
+        <v>166</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>192</v>
+        <v>167</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>73</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -4595,7 +4620,7 @@
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G37" t="s" s="2">
         <v>79</v>
@@ -4610,15 +4635,17 @@
         <v>73</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>108</v>
+        <v>169</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N37" s="2"/>
+        <v>171</v>
+      </c>
+      <c r="N37" t="s" s="2">
+        <v>172</v>
+      </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>73</v>
@@ -4667,10 +4694,10 @@
         <v>73</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="AG37" t="s" s="2">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AH37" t="s" s="2">
         <v>79</v>
@@ -4679,6 +4706,306 @@
         <v>73</v>
       </c>
       <c r="AJ37" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G38" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K38" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="L38" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="M38" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="P38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q38" s="2"/>
+      <c r="R38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF38" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="AG38" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH38" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI38" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ38" t="s" s="2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="B39" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G39" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K39" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="L39" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="M39" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q39" s="2"/>
+      <c r="R39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF39" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="AG39" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH39" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI39" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ39" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="B40" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G40" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K40" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="M40" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2"/>
+      <c r="P40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q40" s="2"/>
+      <c r="R40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF40" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="AG40" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH40" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI40" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ40" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>